<commit_message>
updated webapp and mdl
</commit_message>
<xml_diff>
--- a/InputData/elec/RQSD/RPS Qualifying Source Definitions.xlsx
+++ b/InputData/elec/RQSD/RPS Qualifying Source Definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\RMI\RMI_all_states\PA\elec\RQSD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E9EF0904-D180-4CD5-BDF6-6D201FFECD20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CAC54B43-53D1-4EBC-BFB3-E91557C44EE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="675" windowWidth="15525" windowHeight="16470" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="17160" windowHeight="12645" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -667,7 +667,7 @@
         <v>62</v>
       </c>
       <c r="C1" s="5">
-        <v>45344</v>
+        <v>45345</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2562,97 +2562,127 @@
         <v>32</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C19">
-        <v>1</v>
+        <f>B19</f>
+        <v>0</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <f t="shared" ref="D19:AF22" si="2">C19</f>
+        <v>0</v>
       </c>
       <c r="E19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="H19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="J19">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="K19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="L19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="M19">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="N19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="O19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="P19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="Q19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="R19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="S19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="T19">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="V19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="W19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="X19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="Y19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="Z19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AA19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AB19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AC19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AD19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AE19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AF19">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:32" x14ac:dyDescent="0.25">
@@ -2660,97 +2690,127 @@
         <v>33</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <f t="shared" ref="C20:R22" si="3">B20</f>
+        <v>0</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="E20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="F20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="H20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="J20">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="L20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="M20">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="O20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="P20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="Q20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="R20">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="S20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="T20">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="V20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="W20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="X20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="Y20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="Z20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AA20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AB20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AC20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AD20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AE20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AF20">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:32" x14ac:dyDescent="0.25">
@@ -2758,97 +2818,127 @@
         <v>34</v>
       </c>
       <c r="B21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="I21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="J21">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="K21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="L21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="M21">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="N21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="O21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="P21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="Q21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="R21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="S21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="T21">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="V21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="W21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="X21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="Y21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="Z21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AA21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AB21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AC21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AD21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AE21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AF21">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:32" x14ac:dyDescent="0.25">
@@ -2856,97 +2946,127 @@
         <v>35</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="E22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="J22">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="K22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="L22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="M22">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="N22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="O22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="P22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="Q22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="R22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="S22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="T22">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="V22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="W22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="X22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="Y22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="Z22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AA22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AB22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AC22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AD22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AE22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
       <c r="AF22">
-        <v>1</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:32" x14ac:dyDescent="0.25">
@@ -3437,7 +3557,7 @@
       </c>
       <c r="B19">
         <f>IFERROR(INDEX(Sheet1!$C$2:$AF$25,MATCH($A19,Sheet1!$A$2:$A$25,0),MATCH(About!$B$1,Sheet1!$C$1:$AF$1,0)),Sheet1!B19)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3446,7 +3566,7 @@
       </c>
       <c r="B20">
         <f>IFERROR(INDEX(Sheet1!$C$2:$AF$25,MATCH($A20,Sheet1!$A$2:$A$25,0),MATCH(About!$B$1,Sheet1!$C$1:$AF$1,0)),Sheet1!B20)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -3455,7 +3575,7 @@
       </c>
       <c r="B21">
         <f>IFERROR(INDEX(Sheet1!$C$2:$AF$25,MATCH($A21,Sheet1!$A$2:$A$25,0),MATCH(About!$B$1,Sheet1!$C$1:$AF$1,0)),Sheet1!B21)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3464,7 +3584,7 @@
       </c>
       <c r="B22">
         <f>IFERROR(INDEX(Sheet1!$C$2:$AF$25,MATCH($A22,Sheet1!$A$2:$A$25,0),MATCH(About!$B$1,Sheet1!$C$1:$AF$1,0)),Sheet1!B22)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>